<commit_message>
added again vapt issues
</commit_message>
<xml_diff>
--- a/docs/Retest_Results_BGauss_Response_31.10.2026.xlsx
+++ b/docs/Retest_Results_BGauss_Response_31.10.2026.xlsx
@@ -708,7 +708,7 @@
       <c r="G3" s="24" t="n"/>
       <c r="H3" s="24" t="n"/>
     </row>
-    <row r="4" ht="380" customHeight="1" s="20">
+    <row r="4" ht="400" customHeight="1" s="20">
       <c r="A4" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">DMS-03 </t>
@@ -736,14 +736,15 @@
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>Thank you. Your evidence of 30.10.2026 (POST /api/customers with another dealerId -&gt; HTTP 403 'You are not allowed to access another dealer's data.') confirms that creating a customer under another dealer is blocked. The remaining point - searching another dealer's customer by chassis number - was valid. Cause: the New Job Card wizard's chassis lookup (GET /api/jobcards/vehicle-lookup) first searches the sale bills of the caller's own dealer only; when that found nothing it fell back to an older sales table (DMS_VehicleSales) by chassis number alone, which has no dealer filter, and returned the customer of a vehicle sold by another dealer. This was a defect, not intended behaviour.</t>
+          <t>Thank you. Your evidence of 30.10.2026 (POST /api/customers with another dealerId -&gt; HTTP 403 'You are not allowed to access another dealer's data.') confirms that creating a customer under another dealer is blocked. The remaining point - searching another dealer's customer by chassis number - was valid. Cause: the New Job Card wizard's chassis lookup (GET /api/jobcards/vehicle-lookup) first searches the sale bills of the caller's own dealer only; when that found nothing it fell back to an older sales table (DMS_VehicleSales) by chassis number alone, which has no dealer filter, and returned the customer of a vehicle sold by another dealer. This was a defect, not intended behaviour. A second cause was found while re-testing on the live site: the lookup is scoped by a dealerId parameter, and our ownership filter forced that parameter to the caller's dealer only when it was present in the request - when it was left out, the lookup ran with no dealer filter at all.</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
         <is>
           <t>1. The fallback now ignores a sale row that belongs to another dealer (matched on dealer code, or the location code that starts with it) - the same rule the main lookup already applied. A vehicle sold by another dealer is not found and the wizard falls back to manual entry.
 2. A dealer login whose dealer has no BAPL dealer code used to be searched with no dealer filter; it now gets 'not found' / an empty list.
-3. CorporateAdmin and SystemAdmin are unchanged. Deployed on [DD.MM.YYYY HH:MM IST].</t>
+3. A dealerId that is left out, empty or null is now forced to the caller's own dealer for every action, and another dealer's id is refused with HTTP 403 (the filter used to handle only a dealerId that was present).
+4. CorporateAdmin and SystemAdmin are unchanged. Deployed on [DD.MM.YYYY HH:MM IST].</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">

</xml_diff>